<commit_message>
Fix Render deployment: gunicorn binding, CORS, DATABASE_URL; add multimedia fields, dashboard, reports, approvals, profile, classification, and enhanced search
</commit_message>
<xml_diff>
--- a/MEDICINAL PLANTS/plant_names.xlsx
+++ b/MEDICINAL PLANTS/plant_names.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hp\OneDrive\Desktop\MEDICINAL PLANTS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GIDEON\Desktop\projects\Herbal_Medicine\MEDICINAL PLANTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D95DF20-1EC0-459A-867C-0667A282A619}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="17256" windowHeight="5928"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,6 +20,9 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -1322,7 +1326,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1661,18 +1665,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D148"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="26.5546875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="35.5546875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="26.53125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="35.53125" style="1" customWidth="1"/>
     <col min="3" max="3" width="26.6640625" style="1" customWidth="1"/>
     <col min="4" max="4" width="255.6640625" style="1" customWidth="1"/>
-    <col min="5" max="16384" width="8.88671875" style="1"/>
+    <col min="5" max="16384" width="8.86328125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" s="2" customFormat="1" ht="17.25" x14ac:dyDescent="0.45">
       <c r="A1" s="2" t="s">
         <v>427</v>
       </c>
@@ -1686,7 +1690,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1700,7 +1704,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1714,7 +1718,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -1728,7 +1732,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
@@ -1742,7 +1746,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" s="1" t="s">
         <v>11</v>
       </c>
@@ -1756,7 +1760,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" s="1" t="s">
         <v>13</v>
       </c>
@@ -1770,7 +1774,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" s="1" t="s">
         <v>16</v>
       </c>
@@ -1784,7 +1788,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" s="1" t="s">
         <v>18</v>
       </c>
@@ -1798,7 +1802,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" s="1" t="s">
         <v>20</v>
       </c>
@@ -1812,7 +1816,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" s="1" t="s">
         <v>22</v>
       </c>
@@ -1826,7 +1830,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" s="1" t="s">
         <v>24</v>
       </c>
@@ -1840,7 +1844,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" s="1" t="s">
         <v>26</v>
       </c>
@@ -1854,7 +1858,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" s="1" t="s">
         <v>28</v>
       </c>
@@ -1868,7 +1872,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" s="1" t="s">
         <v>22</v>
       </c>
@@ -1882,7 +1886,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" s="1" t="s">
         <v>22</v>
       </c>
@@ -1896,7 +1900,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A17" s="1" t="s">
         <v>22</v>
       </c>
@@ -1910,7 +1914,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A18" s="1" t="s">
         <v>33</v>
       </c>
@@ -1924,7 +1928,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A19" s="1" t="s">
         <v>35</v>
       </c>
@@ -1938,7 +1942,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A20" s="1" t="s">
         <v>37</v>
       </c>
@@ -1952,7 +1956,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A21" s="1" t="s">
         <v>39</v>
       </c>
@@ -1966,7 +1970,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A22" s="1" t="s">
         <v>22</v>
       </c>
@@ -1980,7 +1984,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A23" s="1" t="s">
         <v>42</v>
       </c>
@@ -1994,7 +1998,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A24" s="1" t="s">
         <v>44</v>
       </c>
@@ -2008,7 +2012,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A25" s="1" t="s">
         <v>46</v>
       </c>
@@ -2022,7 +2026,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A26" s="1" t="s">
         <v>48</v>
       </c>
@@ -2036,7 +2040,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A27" s="1" t="s">
         <v>50</v>
       </c>
@@ -2050,7 +2054,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A28" s="1" t="s">
         <v>52</v>
       </c>
@@ -2064,7 +2068,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A29" s="1" t="s">
         <v>54</v>
       </c>
@@ -2078,7 +2082,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A30" s="1" t="s">
         <v>56</v>
       </c>
@@ -2092,7 +2096,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A31" s="1" t="s">
         <v>58</v>
       </c>
@@ -2106,7 +2110,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A32" s="1" t="s">
         <v>60</v>
       </c>
@@ -2120,7 +2124,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A33" s="1" t="s">
         <v>62</v>
       </c>
@@ -2134,7 +2138,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A34" s="1" t="s">
         <v>64</v>
       </c>
@@ -2148,7 +2152,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A35" s="1" t="s">
         <v>66</v>
       </c>
@@ -2162,7 +2166,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A36" s="1" t="s">
         <v>68</v>
       </c>
@@ -2176,7 +2180,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A37" s="1" t="s">
         <v>70</v>
       </c>
@@ -2190,7 +2194,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A38" s="1" t="s">
         <v>72</v>
       </c>
@@ -2204,7 +2208,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A39" s="1" t="s">
         <v>74</v>
       </c>
@@ -2218,7 +2222,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A40" s="1" t="s">
         <v>76</v>
       </c>
@@ -2232,7 +2236,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A41" s="1" t="s">
         <v>78</v>
       </c>
@@ -2246,7 +2250,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A42" s="1" t="s">
         <v>80</v>
       </c>
@@ -2260,7 +2264,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A43" s="1" t="s">
         <v>82</v>
       </c>
@@ -2274,7 +2278,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A44" s="1" t="s">
         <v>84</v>
       </c>
@@ -2288,7 +2292,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A45" s="1" t="s">
         <v>87</v>
       </c>
@@ -2302,7 +2306,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A46" s="1" t="s">
         <v>89</v>
       </c>
@@ -2316,7 +2320,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A47" s="1" t="s">
         <v>91</v>
       </c>
@@ -2330,7 +2334,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A48" s="1" t="s">
         <v>93</v>
       </c>
@@ -2344,7 +2348,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A49" s="1" t="s">
         <v>95</v>
       </c>
@@ -2358,7 +2362,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A50" s="1" t="s">
         <v>97</v>
       </c>
@@ -2372,7 +2376,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A51" s="1" t="s">
         <v>99</v>
       </c>
@@ -2386,7 +2390,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A52" s="1" t="s">
         <v>74</v>
       </c>
@@ -2400,7 +2404,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A53" s="1" t="s">
         <v>102</v>
       </c>
@@ -2414,7 +2418,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A54" s="1" t="s">
         <v>104</v>
       </c>
@@ -2428,7 +2432,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A55" s="1" t="s">
         <v>106</v>
       </c>
@@ -2442,7 +2446,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A56" s="1" t="s">
         <v>108</v>
       </c>
@@ -2456,7 +2460,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A57" s="1" t="s">
         <v>110</v>
       </c>
@@ -2470,7 +2474,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A58" s="1" t="s">
         <v>112</v>
       </c>
@@ -2484,7 +2488,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A59" s="1" t="s">
         <v>114</v>
       </c>
@@ -2498,7 +2502,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A60" s="1" t="s">
         <v>116</v>
       </c>
@@ -2512,7 +2516,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A61" s="1" t="s">
         <v>118</v>
       </c>
@@ -2526,7 +2530,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A62" s="1" t="s">
         <v>120</v>
       </c>
@@ -2540,7 +2544,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A63" s="1" t="s">
         <v>122</v>
       </c>
@@ -2554,7 +2558,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A64" s="1" t="s">
         <v>124</v>
       </c>
@@ -2568,7 +2572,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A65" s="1" t="s">
         <v>126</v>
       </c>
@@ -2582,7 +2586,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="66" spans="1:4" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:4" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A66" s="1" t="s">
         <v>128</v>
       </c>
@@ -2596,7 +2600,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A67" s="1" t="s">
         <v>130</v>
       </c>
@@ -2610,7 +2614,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A68" s="1" t="s">
         <v>132</v>
       </c>
@@ -2624,7 +2628,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A69" s="1" t="s">
         <v>134</v>
       </c>
@@ -2638,7 +2642,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A70" s="1" t="s">
         <v>136</v>
       </c>
@@ -2652,7 +2656,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A71" s="1" t="s">
         <v>138</v>
       </c>
@@ -2666,7 +2670,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A72" s="1" t="s">
         <v>140</v>
       </c>
@@ -2680,7 +2684,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A73" s="1" t="s">
         <v>142</v>
       </c>
@@ -2694,7 +2698,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A74" s="1" t="s">
         <v>143</v>
       </c>
@@ -2708,7 +2712,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A75" s="1" t="s">
         <v>145</v>
       </c>
@@ -2722,7 +2726,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A76" s="1" t="s">
         <v>147</v>
       </c>
@@ -2733,7 +2737,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A77" s="1" t="s">
         <v>149</v>
       </c>
@@ -2744,7 +2748,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A78" s="1" t="s">
         <v>151</v>
       </c>
@@ -2758,7 +2762,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A79" s="1" t="s">
         <v>153</v>
       </c>
@@ -2772,7 +2776,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A80" s="1" t="s">
         <v>155</v>
       </c>
@@ -2786,7 +2790,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A81" s="1" t="s">
         <v>157</v>
       </c>
@@ -2800,7 +2804,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A82" s="1" t="s">
         <v>159</v>
       </c>
@@ -2814,7 +2818,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A83" s="1" t="s">
         <v>161</v>
       </c>
@@ -2828,7 +2832,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A84" s="1" t="s">
         <v>163</v>
       </c>
@@ -2842,7 +2846,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A85" s="1" t="s">
         <v>165</v>
       </c>
@@ -2856,7 +2860,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A86" s="1" t="s">
         <v>167</v>
       </c>
@@ -2870,7 +2874,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A87" s="1" t="s">
         <v>169</v>
       </c>
@@ -2884,7 +2888,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A88" s="1" t="s">
         <v>170</v>
       </c>
@@ -2898,7 +2902,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A89" s="1" t="s">
         <v>172</v>
       </c>
@@ -2912,7 +2916,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A90" s="1" t="s">
         <v>174</v>
       </c>
@@ -2926,7 +2930,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A91" s="1" t="s">
         <v>176</v>
       </c>
@@ -2940,7 +2944,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A92" s="1" t="s">
         <v>178</v>
       </c>
@@ -2954,7 +2958,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A93" s="1" t="s">
         <v>180</v>
       </c>
@@ -2968,7 +2972,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A94" s="1" t="s">
         <v>182</v>
       </c>
@@ -2982,7 +2986,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A95" s="1" t="s">
         <v>184</v>
       </c>
@@ -2996,7 +3000,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A96" s="1" t="s">
         <v>186</v>
       </c>
@@ -3010,7 +3014,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A97" s="1" t="s">
         <v>184</v>
       </c>
@@ -3024,7 +3028,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A98" s="1" t="s">
         <v>186</v>
       </c>
@@ -3035,7 +3039,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A99" s="1" t="s">
         <v>188</v>
       </c>
@@ -3049,7 +3053,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A100" s="1" t="s">
         <v>190</v>
       </c>
@@ -3063,7 +3067,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A101" s="1" t="s">
         <v>192</v>
       </c>
@@ -3077,7 +3081,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A102" s="1" t="s">
         <v>194</v>
       </c>
@@ -3091,7 +3095,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A103" s="1" t="s">
         <v>196</v>
       </c>
@@ -3105,7 +3109,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A104" s="1" t="s">
         <v>198</v>
       </c>
@@ -3119,7 +3123,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A105" s="1" t="s">
         <v>200</v>
       </c>
@@ -3133,7 +3137,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A106" s="1" t="s">
         <v>202</v>
       </c>
@@ -3147,7 +3151,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A107" s="1" t="s">
         <v>204</v>
       </c>
@@ -3161,7 +3165,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A108" s="1" t="s">
         <v>206</v>
       </c>
@@ -3175,7 +3179,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A109" s="1" t="s">
         <v>208</v>
       </c>
@@ -3189,7 +3193,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A110" s="1" t="s">
         <v>210</v>
       </c>
@@ -3203,7 +3207,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A111" s="1" t="s">
         <v>210</v>
       </c>
@@ -3214,7 +3218,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A112" s="1" t="s">
         <v>212</v>
       </c>
@@ -3228,7 +3232,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A113" s="1" t="s">
         <v>214</v>
       </c>
@@ -3242,7 +3246,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A114" s="1" t="s">
         <v>216</v>
       </c>
@@ -3253,7 +3257,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A115" s="1" t="s">
         <v>218</v>
       </c>
@@ -3267,7 +3271,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A116" s="1" t="s">
         <v>220</v>
       </c>
@@ -3281,7 +3285,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A117" s="1" t="s">
         <v>222</v>
       </c>
@@ -3295,7 +3299,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A118" s="1" t="s">
         <v>224</v>
       </c>
@@ -3309,7 +3313,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A119" s="1" t="s">
         <v>226</v>
       </c>
@@ -3323,7 +3327,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A120" s="1" t="s">
         <v>228</v>
       </c>
@@ -3337,7 +3341,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A121" s="1" t="s">
         <v>230</v>
       </c>
@@ -3351,7 +3355,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A122" s="1" t="s">
         <v>232</v>
       </c>
@@ -3365,7 +3369,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A123" s="1" t="s">
         <v>234</v>
       </c>
@@ -3379,7 +3383,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A124" s="1" t="s">
         <v>236</v>
       </c>
@@ -3393,7 +3397,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A125" s="1" t="s">
         <v>238</v>
       </c>
@@ -3407,7 +3411,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A126" s="1" t="s">
         <v>240</v>
       </c>
@@ -3421,7 +3425,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A127" s="1" t="s">
         <v>242</v>
       </c>
@@ -3435,7 +3439,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A128" s="1" t="s">
         <v>244</v>
       </c>
@@ -3449,7 +3453,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A129" s="1" t="s">
         <v>246</v>
       </c>
@@ -3463,7 +3467,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A130" s="1" t="s">
         <v>248</v>
       </c>
@@ -3477,7 +3481,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A131" s="1" t="s">
         <v>250</v>
       </c>
@@ -3491,7 +3495,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A132" s="1" t="s">
         <v>252</v>
       </c>
@@ -3505,7 +3509,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A133" s="1" t="s">
         <v>254</v>
       </c>
@@ -3519,7 +3523,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A134" s="1" t="s">
         <v>256</v>
       </c>
@@ -3533,7 +3537,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A135" s="1" t="s">
         <v>258</v>
       </c>
@@ -3547,7 +3551,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A136" s="1" t="s">
         <v>260</v>
       </c>
@@ -3561,7 +3565,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A137" s="1" t="s">
         <v>262</v>
       </c>
@@ -3572,7 +3576,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A138" s="1" t="s">
         <v>264</v>
       </c>
@@ -3586,7 +3590,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A139" s="1" t="s">
         <v>266</v>
       </c>
@@ -3600,7 +3604,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A140" s="1" t="s">
         <v>268</v>
       </c>
@@ -3614,7 +3618,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A141" s="1" t="s">
         <v>270</v>
       </c>
@@ -3628,7 +3632,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A142" s="1" t="s">
         <v>272</v>
       </c>
@@ -3639,7 +3643,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A143" s="1" t="s">
         <v>274</v>
       </c>
@@ -3653,7 +3657,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A144" s="1" t="s">
         <v>276</v>
       </c>
@@ -3667,7 +3671,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A145" s="1" t="s">
         <v>74</v>
       </c>
@@ -3681,7 +3685,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A146" s="1" t="s">
         <v>279</v>
       </c>
@@ -3695,7 +3699,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A147" s="1" t="s">
         <v>281</v>
       </c>
@@ -3709,7 +3713,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A148" s="1" t="s">
         <v>283</v>
       </c>
@@ -3722,9 +3726,9 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D26"/>
-    <hyperlink ref="D140"/>
-    <hyperlink ref="D66"/>
+    <hyperlink ref="D26" display="https://www.google.com/imgres?q=Hibiscus%20surattensis%20L&amp;imgurl=https%3A%2F%2Flive.staticflickr.com%2F2684%2F4302824951_282a641c57_b.jpg&amp;imgrefurl=https%3A%2F%2Fwww.flickr.com%2Fphotos%2Fbuoichieu%2F4302824951&amp;docid=Dugv6nJghwTVZM&amp;tbnid=2LyhC1RDeJ1UaM&amp;v" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="D140" display="https://www.google.com/imgres?q=Flueggea%20virosa%0D%0A&amp;imgurl=https%3A%2F%2Flive.staticflickr.com%2F8656%2F16429510476_b2afd6eec0_b.jpg&amp;imgrefurl=https%3A%2F%2Fwww.flickr.com%2Fphotos%2Fberniedup%2F16429510476&amp;docid=hjrkrkyi-3PURM&amp;tbnid=hMuoI2mywJyExM&amp;ve" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="D66" display="https://www.google.com/imgres?q=Ficus%20natalensis%0D%0A&amp;imgurl=https%3A%2F%2Flive.staticflickr.com%2F337%2F20226385596_ef87a91f9c_b.jpg&amp;imgrefurl=https%3A%2F%2Fwww.flickr.com%2Fphotos%2F89906643%40N06%2F20226385596&amp;docid=eh7LCaY08rfklM&amp;tbnid=z_FQ03vYRsqj" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>